<commit_message>
Conflict battery item validation checks, review artifacts, similarity scoring.
</commit_message>
<xml_diff>
--- a/data/battery/workbooks/CB_type10_privacy_vs_care.xlsx
+++ b/data/battery/workbooks/CB_type10_privacy_vs_care.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\GitHub\llm-conflict-probing\data\battery\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C74CF70D-02E1-4DC6-A7F3-4361E62514AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92E80C2A-348A-471D-8C6C-B036C98A228A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,12 +19,11 @@
     <sheet name="Type_summary" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="193">
   <si>
     <t>Conflict Battery — Type 10: privacy (refuse-pole) vs. care (refusal family)</t>
   </si>
@@ -597,9 +596,6 @@
   </si>
   <si>
     <t>Don't tell anyone I'm unwell or struggling</t>
-  </si>
-  <si>
-    <t>edit</t>
   </si>
   <si>
     <t>remove explicit requests to not tell anyone</t>
@@ -1377,7 +1373,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:14" ht="87" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
         <v>58</v>
       </c>
@@ -1412,14 +1408,14 @@
       <c r="L2" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="N2" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="N2" s="8" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
+    </row>
+    <row r="3" spans="1:14" ht="87" x14ac:dyDescent="0.4">
       <c r="A3" s="6" t="s">
         <v>58</v>
       </c>
@@ -1454,14 +1450,14 @@
       <c r="L3" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="M3" s="10" t="s">
-        <v>191</v>
+      <c r="M3" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="87" x14ac:dyDescent="0.4">
       <c r="A4" s="6" t="s">
         <v>58</v>
       </c>
@@ -1498,14 +1494,14 @@
       <c r="L4" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="M4" s="10" t="s">
-        <v>191</v>
+      <c r="M4" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="87" x14ac:dyDescent="0.4">
       <c r="A5" s="6" t="s">
         <v>58</v>
       </c>
@@ -1542,11 +1538,11 @@
       <c r="L5" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="M5" s="10" t="s">
-        <v>191</v>
+      <c r="M5" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="87" x14ac:dyDescent="0.4">
@@ -1584,11 +1580,11 @@
       <c r="L6" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="M6" s="10" t="s">
-        <v>191</v>
+      <c r="M6" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="87" x14ac:dyDescent="0.4">
@@ -1626,11 +1622,11 @@
       <c r="L7" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="M7" s="10" t="s">
-        <v>191</v>
+      <c r="M7" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N7" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="87" x14ac:dyDescent="0.4">
@@ -1670,11 +1666,11 @@
       <c r="L8" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="M8" s="10" t="s">
-        <v>191</v>
+      <c r="M8" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="87" x14ac:dyDescent="0.4">
@@ -1714,14 +1710,14 @@
       <c r="L9" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="M9" s="10" t="s">
-        <v>191</v>
+      <c r="M9" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N9" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
       <c r="A10" s="6" t="s">
         <v>98</v>
       </c>
@@ -1756,14 +1752,14 @@
       <c r="L10" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="M10" s="10" t="s">
-        <v>191</v>
+      <c r="M10" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
       <c r="A11" s="6" t="s">
         <v>98</v>
       </c>
@@ -1798,14 +1794,14 @@
       <c r="L11" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="M11" s="10" t="s">
-        <v>191</v>
+      <c r="M11" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N11" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
       <c r="A12" s="6" t="s">
         <v>98</v>
       </c>
@@ -1842,14 +1838,14 @@
       <c r="L12" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="M12" s="10" t="s">
-        <v>191</v>
+      <c r="M12" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N12" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
       <c r="A13" s="6" t="s">
         <v>98</v>
       </c>
@@ -1886,11 +1882,11 @@
       <c r="L13" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="M13" s="10" t="s">
-        <v>191</v>
+      <c r="M13" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
@@ -1928,11 +1924,11 @@
       <c r="L14" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="M14" s="10" t="s">
-        <v>191</v>
+      <c r="M14" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
@@ -1970,11 +1966,11 @@
       <c r="L15" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="M15" s="10" t="s">
-        <v>191</v>
+      <c r="M15" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
@@ -2014,11 +2010,11 @@
       <c r="L16" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="M16" s="10" t="s">
-        <v>191</v>
+      <c r="M16" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N16" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
@@ -2058,14 +2054,14 @@
       <c r="L17" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="M17" s="10" t="s">
-        <v>191</v>
+      <c r="M17" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="87" x14ac:dyDescent="0.4">
       <c r="A18" s="6" t="s">
         <v>124</v>
       </c>
@@ -2100,14 +2096,14 @@
       <c r="L18" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="M18" s="10" t="s">
-        <v>191</v>
+      <c r="M18" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N18" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="87" x14ac:dyDescent="0.4">
       <c r="A19" s="6" t="s">
         <v>124</v>
       </c>
@@ -2142,14 +2138,14 @@
       <c r="L19" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="M19" s="10" t="s">
-        <v>191</v>
+      <c r="M19" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="87" x14ac:dyDescent="0.4">
       <c r="A20" s="6" t="s">
         <v>124</v>
       </c>
@@ -2186,14 +2182,14 @@
       <c r="L20" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="M20" s="10" t="s">
-        <v>191</v>
+      <c r="M20" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N20" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="87" x14ac:dyDescent="0.4">
       <c r="A21" s="6" t="s">
         <v>124</v>
       </c>
@@ -2230,14 +2226,14 @@
       <c r="L21" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="M21" s="10" t="s">
-        <v>191</v>
+      <c r="M21" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
       <c r="A22" s="6" t="s">
         <v>135</v>
       </c>
@@ -2272,14 +2268,14 @@
       <c r="L22" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="M22" s="10" t="s">
-        <v>191</v>
+      <c r="M22" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N22" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
       <c r="A23" s="6" t="s">
         <v>135</v>
       </c>
@@ -2314,14 +2310,14 @@
       <c r="L23" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="M23" s="10" t="s">
-        <v>191</v>
+      <c r="M23" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
       <c r="A24" s="6" t="s">
         <v>135</v>
       </c>
@@ -2358,14 +2354,14 @@
       <c r="L24" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="M24" s="10" t="s">
-        <v>191</v>
+      <c r="M24" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N24" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="111.9" x14ac:dyDescent="0.4">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="99.45" x14ac:dyDescent="0.4">
       <c r="A25" s="6" t="s">
         <v>135</v>
       </c>
@@ -2402,11 +2398,11 @@
       <c r="L25" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="M25" s="10" t="s">
-        <v>191</v>
+      <c r="M25" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>